<commit_message>
Update Clean epitope sequences
</commit_message>
<xml_diff>
--- a/Clean epitope sequences/cleaning_summary.xlsx
+++ b/Clean epitope sequences/cleaning_summary.xlsx
@@ -453,16 +453,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2933</v>
+        <v>2877</v>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>0.9865455768583922</v>
+        <v>0.9893397524071527</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0.0134544231416078</v>
+        <v>0.01066024759284732</v>
       </c>
     </row>
     <row r="3">
@@ -475,13 +475,13 @@
         <v>2169</v>
       </c>
       <c r="C3" t="n">
-        <v>256</v>
+        <v>175</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0.8944329896907216</v>
+        <v>0.9253412969283277</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0.1055670103092784</v>
+        <v>0.07465870307167236</v>
       </c>
     </row>
     <row r="4">
@@ -491,16 +491,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2009</v>
+        <v>1944</v>
       </c>
       <c r="C4" t="n">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.9480887210948561</v>
+        <v>0.9515418502202643</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.05191127890514394</v>
+        <v>0.04845814977973568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>